<commit_message>
Add management learning pipeline
</commit_message>
<xml_diff>
--- a/exports/daily_trades_2026-07-20.xlsx
+++ b/exports/daily_trades_2026-07-20.xlsx
@@ -485,40 +485,28 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>11.10000038146973</v>
+        <v>11.01500034332275</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Iron Condor</t>
+          <t>Short Strangle</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="E2" t="n">
-        <v>-9.909913006003679</v>
-      </c>
-      <c r="F2" t="n">
-        <v>-32.43243475450276</v>
+        <v>-9.214710047086317</v>
       </c>
       <c r="G2" t="n">
-        <v>3.603600043095767</v>
-      </c>
-      <c r="H2" t="n">
-        <v>26.12612179159486</v>
+        <v>4.403083445850742</v>
       </c>
       <c r="I2" t="n">
         <v>10</v>
       </c>
-      <c r="J2" t="n">
-        <v>7.5</v>
-      </c>
       <c r="K2" t="n">
         <v>11.5</v>
       </c>
-      <c r="L2" t="n">
-        <v>14</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -527,39 +515,27 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>148.6900024414062</v>
+        <v>144.7100067138672</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Iron Condor</t>
+          <t>Short Strangle</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="E3" t="n">
-        <v>-7.189456093807534</v>
-      </c>
-      <c r="F3" t="n">
-        <v>-10.55215695997392</v>
+        <v>-6.709975995693673</v>
       </c>
       <c r="G3" t="n">
-        <v>7.606427717324604</v>
-      </c>
-      <c r="H3" t="n">
-        <v>10.969128583491</v>
+        <v>7.1107683012406</v>
       </c>
       <c r="I3" t="n">
-        <v>138</v>
-      </c>
-      <c r="J3" t="n">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="K3" t="n">
-        <v>160</v>
-      </c>
-      <c r="L3" t="n">
-        <v>165</v>
+        <v>155</v>
       </c>
     </row>
     <row r="4">
@@ -569,39 +545,27 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>203.8950042724609</v>
+        <v>202.2200012207031</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Iron Condor</t>
+          <t>Short Strangle</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="E4" t="n">
-        <v>-6.814784070870772</v>
-      </c>
-      <c r="F4" t="n">
-        <v>-11.7192691197723</v>
+        <v>-6.042924115783288</v>
       </c>
       <c r="G4" t="n">
-        <v>6.672549813608475</v>
-      </c>
-      <c r="H4" t="n">
-        <v>11.57703486251</v>
+        <v>6.319849026876811</v>
       </c>
       <c r="I4" t="n">
         <v>190</v>
       </c>
-      <c r="J4" t="n">
-        <v>180</v>
-      </c>
       <c r="K4" t="n">
-        <v>217.5</v>
-      </c>
-      <c r="L4" t="n">
-        <v>227.5</v>
+        <v>215</v>
       </c>
     </row>
     <row r="5">
@@ -611,40 +575,28 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>76.02999877929688</v>
+        <v>75.54000091552734</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Iron Condor</t>
+          <t>Short Strangle</t>
         </is>
       </c>
       <c r="D5" t="n">
         <v>38</v>
       </c>
       <c r="E5" t="n">
-        <v>-6.615808049528149</v>
-      </c>
-      <c r="F5" t="n">
-        <v>-13.19215959533603</v>
+        <v>-7.333863977209177</v>
       </c>
       <c r="G5" t="n">
-        <v>9.16743566041076</v>
-      </c>
-      <c r="H5" t="n">
-        <v>15.74378720621863</v>
+        <v>9.875561284166267</v>
       </c>
       <c r="I5" t="n">
-        <v>71</v>
-      </c>
-      <c r="J5" t="n">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="K5" t="n">
         <v>83</v>
       </c>
-      <c r="L5" t="n">
-        <v>88</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -653,39 +605,27 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>35.81000137329102</v>
+        <v>35.66500091552734</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Iron Condor</t>
+          <t>Short Strangle</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="E6" t="n">
-        <v>-7.846973654088885</v>
-      </c>
-      <c r="F6" t="n">
-        <v>-14.82826352877913</v>
+        <v>-7.472314165473892</v>
       </c>
       <c r="G6" t="n">
-        <v>8.908122045167666</v>
-      </c>
-      <c r="H6" t="n">
-        <v>14.49315394491986</v>
+        <v>5.1450975392342</v>
       </c>
       <c r="I6" t="n">
         <v>33</v>
       </c>
-      <c r="J6" t="n">
-        <v>30.5</v>
-      </c>
       <c r="K6" t="n">
-        <v>39</v>
-      </c>
-      <c r="L6" t="n">
-        <v>41</v>
+        <v>37.5</v>
       </c>
     </row>
     <row r="7">
@@ -695,39 +635,27 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>161.1699981689453</v>
+        <v>160.4382019042969</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Iron Condor</t>
+          <t>Short Strangle</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="E7" t="n">
-        <v>-6.930569148010068</v>
-      </c>
-      <c r="F7" t="n">
-        <v>-13.13519787147606</v>
+        <v>-6.506057647369657</v>
       </c>
       <c r="G7" t="n">
-        <v>7.029845479788421</v>
-      </c>
-      <c r="H7" t="n">
-        <v>13.23447420325441</v>
+        <v>5.959801332981063</v>
       </c>
       <c r="I7" t="n">
         <v>150</v>
       </c>
-      <c r="J7" t="n">
-        <v>140</v>
-      </c>
       <c r="K7" t="n">
-        <v>172.5</v>
-      </c>
-      <c r="L7" t="n">
-        <v>182.5</v>
+        <v>170</v>
       </c>
     </row>
     <row r="8">
@@ -737,39 +665,27 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>101.2050018310547</v>
+        <v>102.3199996948242</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Iron Condor</t>
+          <t>Short Strangle</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="E8" t="n">
-        <v>-7.119215158043534</v>
-      </c>
-      <c r="F8" t="n">
-        <v>-12.05968243687101</v>
+        <v>-5.199374228588205</v>
       </c>
       <c r="G8" t="n">
-        <v>4.737906311142392</v>
-      </c>
-      <c r="H8" t="n">
-        <v>9.678373589969858</v>
+        <v>4.573886160217144</v>
       </c>
       <c r="I8" t="n">
-        <v>94</v>
-      </c>
-      <c r="J8" t="n">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="K8" t="n">
-        <v>106</v>
-      </c>
-      <c r="L8" t="n">
-        <v>111</v>
+        <v>107</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add action-based management KNN
</commit_message>
<xml_diff>
--- a/exports/daily_trades_2026-07-20.xlsx
+++ b/exports/daily_trades_2026-07-20.xlsx
@@ -485,7 +485,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>11.01500034332275</v>
+        <v>10.65499973297119</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -493,13 +493,13 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>48</v>
+        <v>72</v>
       </c>
       <c r="E2" t="n">
-        <v>-9.214710047086317</v>
+        <v>-6.147346310524416</v>
       </c>
       <c r="G2" t="n">
-        <v>4.403083445850742</v>
+        <v>7.930551742896919</v>
       </c>
       <c r="I2" t="n">
         <v>10</v>
@@ -515,7 +515,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>144.7100067138672</v>
+        <v>146.1999969482422</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -523,19 +523,19 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>38</v>
+        <v>58</v>
       </c>
       <c r="E3" t="n">
-        <v>-6.709975995693673</v>
+        <v>-7.660736786613764</v>
       </c>
       <c r="G3" t="n">
-        <v>7.1107683012406</v>
+        <v>12.85909948302761</v>
       </c>
       <c r="I3" t="n">
         <v>135</v>
       </c>
       <c r="K3" t="n">
-        <v>155</v>
+        <v>165</v>
       </c>
     </row>
     <row r="4">
@@ -545,7 +545,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>202.2200012207031</v>
+        <v>191.75</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -553,19 +553,19 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>38</v>
+        <v>67</v>
       </c>
       <c r="E4" t="n">
-        <v>-6.042924115783288</v>
+        <v>-13.95045632333768</v>
       </c>
       <c r="G4" t="n">
-        <v>6.319849026876811</v>
+        <v>10.82138200782268</v>
       </c>
       <c r="I4" t="n">
-        <v>190</v>
+        <v>165</v>
       </c>
       <c r="K4" t="n">
-        <v>215</v>
+        <v>212.5</v>
       </c>
     </row>
     <row r="5">
@@ -575,7 +575,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>75.54000091552734</v>
+        <v>83.59999847412109</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -583,19 +583,19 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>38</v>
+        <v>59</v>
       </c>
       <c r="E5" t="n">
-        <v>-7.333863977209177</v>
+        <v>-11.48325197289667</v>
       </c>
       <c r="G5" t="n">
-        <v>9.875561284166267</v>
+        <v>19.61722706365314</v>
       </c>
       <c r="I5" t="n">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="K5" t="n">
-        <v>83</v>
+        <v>100</v>
       </c>
     </row>
     <row r="6">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>35.66500091552734</v>
+        <v>33.16500091552734</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -613,16 +613,16 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>38</v>
+        <v>57</v>
       </c>
       <c r="E6" t="n">
-        <v>-7.472314165473892</v>
+        <v>-8.035582216069326</v>
       </c>
       <c r="G6" t="n">
-        <v>5.1450975392342</v>
+        <v>13.07100547204591</v>
       </c>
       <c r="I6" t="n">
-        <v>33</v>
+        <v>30.5</v>
       </c>
       <c r="K6" t="n">
         <v>37.5</v>
@@ -635,7 +635,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>160.4382019042969</v>
+        <v>173.0599975585938</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -643,19 +643,19 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>38</v>
+        <v>56</v>
       </c>
       <c r="E7" t="n">
-        <v>-6.506057647369657</v>
+        <v>-10.43568578144646</v>
       </c>
       <c r="G7" t="n">
-        <v>5.959801332981063</v>
+        <v>15.56685705619811</v>
       </c>
       <c r="I7" t="n">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="K7" t="n">
-        <v>170</v>
+        <v>200</v>
       </c>
     </row>
     <row r="8">
@@ -665,7 +665,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>102.3199996948242</v>
+        <v>101.75</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -673,19 +673,19 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>38</v>
+        <v>65</v>
       </c>
       <c r="E8" t="n">
-        <v>-5.199374228588205</v>
+        <v>-7.616707616707618</v>
       </c>
       <c r="G8" t="n">
-        <v>4.573886160217144</v>
+        <v>9.090909090909083</v>
       </c>
       <c r="I8" t="n">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="K8" t="n">
-        <v>107</v>
+        <v>111</v>
       </c>
     </row>
   </sheetData>

</xml_diff>